<commit_message>
separate the feature cut from the refit, the drop was the feature cut
</commit_message>
<xml_diff>
--- a/04_Figures/shared/WGCNA/loso_refit/c_data/loso_refit.xlsx
+++ b/04_Figures/shared/WGCNA/loso_refit/c_data/loso_refit.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="39">
   <si>
     <t xml:space="preserve">stage</t>
   </si>
@@ -33,6 +33,9 @@
     <t xml:space="preserve">metric_insample</t>
   </si>
   <si>
+    <t xml:space="preserve">metric_cohort_reduced</t>
+  </si>
+  <si>
     <t xml:space="preserve">metric_loso_refit</t>
   </si>
   <si>
@@ -40,6 +43,12 @@
   </si>
   <si>
     <t xml:space="preserve">drop</t>
+  </si>
+  <si>
+    <t xml:space="preserve">drop_from_features</t>
+  </si>
+  <si>
+    <t xml:space="preserve">drop_from_refit</t>
   </si>
   <si>
     <t xml:space="preserve">F06_prediction</t>
@@ -477,22 +486,31 @@
       <c r="I1" t="s">
         <v>8</v>
       </c>
+      <c r="J1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="B2" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="C2" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="D2" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="E2" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="F2" t="n">
         <v>0.2160515511346</v>
@@ -501,27 +519,36 @@
         <v>-0.14795918367347</v>
       </c>
       <c r="H2" t="n">
+        <v>-0.14795918367347</v>
+      </c>
+      <c r="I2" t="n">
         <v>0.82089552238806</v>
       </c>
-      <c r="I2" t="n">
+      <c r="J2" t="n">
         <v>0.36401073480807</v>
+      </c>
+      <c r="K2" t="n">
+        <v>0.36401073480807</v>
+      </c>
+      <c r="L2" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="B3" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="C3" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="D3" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="E3" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="F3" t="n">
         <v>0.249732775292857</v>
@@ -530,85 +557,112 @@
         <v>-0.14795918367347</v>
       </c>
       <c r="H3" t="n">
+        <v>-0.14795918367347</v>
+      </c>
+      <c r="I3" t="n">
         <v>0.81592039800995</v>
       </c>
-      <c r="I3" t="n">
+      <c r="J3" t="n">
         <v>0.397691958966326</v>
+      </c>
+      <c r="K3" t="n">
+        <v>0.397691958966326</v>
+      </c>
+      <c r="L3" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="B4" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="C4" t="s">
+        <v>18</v>
+      </c>
+      <c r="D4" t="s">
         <v>15</v>
       </c>
-      <c r="D4" t="s">
-        <v>12</v>
-      </c>
       <c r="E4" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="F4" t="n">
         <v>0.309257343662561</v>
       </c>
       <c r="G4" t="n">
+        <v>-0.0779980153842508</v>
+      </c>
+      <c r="H4" t="n">
         <v>-0.207549805410135</v>
       </c>
-      <c r="H4" t="n">
+      <c r="I4" t="n">
         <v>0.338308457711443</v>
       </c>
-      <c r="I4" t="n">
+      <c r="J4" t="n">
         <v>0.516807149072696</v>
+      </c>
+      <c r="K4" t="n">
+        <v>0.387255359046812</v>
+      </c>
+      <c r="L4" t="n">
+        <v>0.129551790025884</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="B5" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="C5" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="D5" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="E5" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="F5" t="n">
         <v>0.214388914026353</v>
       </c>
       <c r="G5" t="n">
+        <v>-0.313415932943927</v>
+      </c>
+      <c r="H5" t="n">
         <v>-0.301514641086706</v>
       </c>
-      <c r="H5" t="n">
+      <c r="I5" t="n">
         <v>0.338308457711443</v>
       </c>
-      <c r="I5" t="n">
+      <c r="J5" t="n">
         <v>0.515903555113059</v>
+      </c>
+      <c r="K5" t="n">
+        <v>0.52780484697028</v>
+      </c>
+      <c r="L5" t="n">
+        <v>-0.0119012918572212</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="B6" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="C6" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="D6" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="E6" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="F6" t="n">
         <v>0.282583392968293</v>
@@ -617,27 +671,36 @@
         <v>-0.159763313609467</v>
       </c>
       <c r="H6" t="n">
+        <v>-0.159763313609467</v>
+      </c>
+      <c r="I6" t="n">
         <v>0.378109452736318</v>
       </c>
-      <c r="I6" t="n">
+      <c r="J6" t="n">
         <v>0.44234670657776</v>
+      </c>
+      <c r="K6" t="n">
+        <v>0.44234670657776</v>
+      </c>
+      <c r="L6" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="B7" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="C7" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="D7" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="E7" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="F7" t="n">
         <v>0.262322625063435</v>
@@ -646,68 +709,95 @@
         <v>-0.159763313609467</v>
       </c>
       <c r="H7" t="n">
+        <v>-0.159763313609467</v>
+      </c>
+      <c r="I7" t="n">
         <v>0.398009950248756</v>
       </c>
-      <c r="I7" t="n">
+      <c r="J7" t="n">
         <v>0.422085938672902</v>
+      </c>
+      <c r="K7" t="n">
+        <v>0.422085938672902</v>
+      </c>
+      <c r="L7" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="B8" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="C8" t="s">
+        <v>22</v>
+      </c>
+      <c r="D8" t="s">
+        <v>15</v>
+      </c>
+      <c r="E8" t="s">
         <v>19</v>
-      </c>
-      <c r="D8" t="s">
-        <v>12</v>
-      </c>
-      <c r="E8" t="s">
-        <v>16</v>
       </c>
       <c r="F8" t="n">
         <v>0.385810185737778</v>
       </c>
       <c r="G8" t="n">
+        <v>-0.0481455557948103</v>
+      </c>
+      <c r="H8" t="n">
         <v>-0.0936150131806179</v>
       </c>
-      <c r="H8" t="n">
+      <c r="I8" t="n">
         <v>0.253731343283582</v>
       </c>
-      <c r="I8" t="n">
+      <c r="J8" t="n">
         <v>0.479425198918396</v>
+      </c>
+      <c r="K8" t="n">
+        <v>0.433955741532588</v>
+      </c>
+      <c r="L8" t="n">
+        <v>0.0454694573858077</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="B9" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="C9" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="D9" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="E9" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="F9" t="n">
         <v>0.36795135249738</v>
       </c>
       <c r="G9" t="n">
+        <v>-0.244478204343245</v>
+      </c>
+      <c r="H9" t="n">
         <v>-0.211204123504218</v>
       </c>
-      <c r="H9" t="n">
+      <c r="I9" t="n">
         <v>0.223880597014925</v>
       </c>
-      <c r="I9" t="n">
+      <c r="J9" t="n">
         <v>0.579155476001598</v>
+      </c>
+      <c r="K9" t="n">
+        <v>0.612429556840625</v>
+      </c>
+      <c r="L9" t="n">
+        <v>-0.0332740808390271</v>
       </c>
     </row>
   </sheetData>
@@ -723,24 +813,24 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="B1" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="C1" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="D1" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="E1" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="B2" t="n">
         <v>0.392848713237482</v>
@@ -757,7 +847,7 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="B3" t="n">
         <v>0.533381687884177</v>
@@ -774,7 +864,7 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="B4" t="n">
         <v>0.456717814398046</v>
@@ -791,7 +881,7 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="B5" t="n">
         <v>0.616283434304412</v>
@@ -808,7 +898,7 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="B6" t="n">
         <v>0.536991779737618</v>
@@ -825,7 +915,7 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="B7" t="n">
         <v>0.853836519990896</v>
@@ -842,7 +932,7 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="B8" t="n">
         <v>0.462187563531427</v>
@@ -859,7 +949,7 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="B9" t="n">
         <v>0.376967366269988</v>
@@ -876,7 +966,7 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="B10" t="n">
         <v>0.497336879208876</v>
@@ -893,7 +983,7 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="B11" t="n">
         <v>0.882277104195404</v>
@@ -910,7 +1000,7 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="B12" t="n">
         <v>0.609363488973251</v>

</xml_diff>